<commit_message>
Updated excel master record
</commit_message>
<xml_diff>
--- a/Dyashin-Training-Master-Tracker-Record.xlsx
+++ b/Dyashin-Training-Master-Tracker-Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dyashin-tutorial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2AF903-10F6-4E71-9CF7-40BB5D6840A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A855CB-F68B-415B-9B17-2479F2D2AD7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{04FCAFE5-9534-4F2F-ACC7-2F9728B33BA2}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="68">
   <si>
     <t>Date</t>
   </si>
@@ -184,6 +184,60 @@
   </si>
   <si>
     <t>CSS Handson practice</t>
+  </si>
+  <si>
+    <t>Assessment</t>
+  </si>
+  <si>
+    <t>Oral assessment take</t>
+  </si>
+  <si>
+    <t>Volunteer</t>
+  </si>
+  <si>
+    <t>Deployed Case Study Project</t>
+  </si>
+  <si>
+    <t>Volunteer Task</t>
+  </si>
+  <si>
+    <t>Find BMI from inputs</t>
+  </si>
+  <si>
+    <t>Assignment Completed 1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assignment Completed 1.2 </t>
+  </si>
+  <si>
+    <t>Assignment Completed 1.3</t>
+  </si>
+  <si>
+    <t>Array Methods Practice</t>
+  </si>
+  <si>
+    <t>2 Array Practice Tasks Completion</t>
+  </si>
+  <si>
+    <t>Completed all the tasks given</t>
+  </si>
+  <si>
+    <t>Task Research on Promise methods</t>
+  </si>
+  <si>
+    <t>Promises Practice</t>
+  </si>
+  <si>
+    <t>Task Complete the Coding Problems give</t>
+  </si>
+  <si>
+    <t>Completed Assignment task 2.1</t>
+  </si>
+  <si>
+    <t>Completed Assignment task 2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task </t>
   </si>
 </sst>
 </file>
@@ -403,66 +457,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="0"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="0"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -780,13 +774,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -799,6 +786,73 @@
         <bottom style="medium">
           <color rgb="FFCCCCCC"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="0"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="0"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
   </dxfs>
@@ -815,17 +869,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41E48F9C-D00C-4230-BFD8-0CECC030125D}" name="Table1" displayName="Table1" ref="A1:H48" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
-  <autoFilter ref="A1:H48" xr:uid="{41E48F9C-D00C-4230-BFD8-0CECC030125D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41E48F9C-D00C-4230-BFD8-0CECC030125D}" name="Table1" displayName="Table1" ref="A1:H59" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+  <autoFilter ref="A1:H59" xr:uid="{41E48F9C-D00C-4230-BFD8-0CECC030125D}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2A26C5F3-F6F5-408A-9023-BEE119F726B8}" name="Date" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{EFAA7E6B-D8D1-4A29-ADAB-AE44D9FE76A7}" name="Topic" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{303C7E96-F438-4232-9E60-7707DD0A5B87}" name="Task" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{10E92546-2CDD-4FAE-94F0-397408FF210F}" name="Type" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{67601539-C4ED-418B-8929-5D508ABA13D6}" name="Status" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{BBA490B7-96CF-45AB-B8F1-4574F85D3560}" name="GitHub" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{562FC09F-63FC-4024-9D5E-4C39B524F673}" name="Deployment" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{3EBF1334-CF4D-4765-B4E7-B511CA7A5D6F}" name="Presentation" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{2A26C5F3-F6F5-408A-9023-BEE119F726B8}" name="Date" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{EFAA7E6B-D8D1-4A29-ADAB-AE44D9FE76A7}" name="Topic" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{303C7E96-F438-4232-9E60-7707DD0A5B87}" name="Task" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{10E92546-2CDD-4FAE-94F0-397408FF210F}" name="Type" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{67601539-C4ED-418B-8929-5D508ABA13D6}" name="Status" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{BBA490B7-96CF-45AB-B8F1-4574F85D3560}" name="GitHub" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{562FC09F-63FC-4024-9D5E-4C39B524F673}" name="Deployment" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{3EBF1334-CF4D-4765-B4E7-B511CA7A5D6F}" name="Presentation" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1128,7 +1182,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C217E04-B9EA-4E6C-A4A3-4C970AA68344}">
-  <dimension ref="A1:Z1014"/>
+  <dimension ref="A1:Z1025"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="20.7109375" style="5" customWidth="1"/>
@@ -1670,11 +1724,21 @@
       <c r="Z14" s="4"/>
     </row>
     <row r="15" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="14"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
+      <c r="A15" s="14">
+        <v>46276</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="7"/>
@@ -1698,11 +1762,21 @@
       <c r="Z15" s="4"/>
     </row>
     <row r="16" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="14"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
+      <c r="A16" s="14">
+        <v>46276</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="7"/>
@@ -1754,11 +1828,21 @@
       <c r="Z17" s="4"/>
     </row>
     <row r="18" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
+      <c r="A18" s="14">
+        <v>46280</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="7"/>
@@ -1782,11 +1866,21 @@
       <c r="Z18" s="4"/>
     </row>
     <row r="19" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
+      <c r="A19" s="14">
+        <v>46280</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="7"/>
@@ -1810,11 +1904,21 @@
       <c r="Z19" s="4"/>
     </row>
     <row r="20" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
+      <c r="A20" s="14">
+        <v>46281</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
       <c r="H20" s="7"/>
@@ -1838,11 +1942,21 @@
       <c r="Z20" s="4"/>
     </row>
     <row r="21" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="14"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
+      <c r="A21" s="14">
+        <v>46281</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="7"/>
@@ -1866,11 +1980,21 @@
       <c r="Z21" s="4"/>
     </row>
     <row r="22" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="14"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
+      <c r="A22" s="14">
+        <v>46282</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="7"/>
@@ -1894,11 +2018,21 @@
       <c r="Z22" s="4"/>
     </row>
     <row r="23" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="14"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
+      <c r="A23" s="14">
+        <v>46283</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="7"/>
@@ -1922,11 +2056,21 @@
       <c r="Z23" s="4"/>
     </row>
     <row r="24" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="14"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
+      <c r="A24" s="14">
+        <v>46283</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="7"/>
@@ -1978,11 +2122,21 @@
       <c r="Z25" s="4"/>
     </row>
     <row r="26" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="14"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
+      <c r="A26" s="14">
+        <v>46286</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="7"/>
@@ -2006,30 +2160,24 @@
       <c r="Z26" s="4"/>
     </row>
     <row r="27" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="9">
-        <v>46289</v>
+      <c r="A27" s="14">
+        <v>46286</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F27" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="7"/>
       <c r="I27" s="4"/>
       <c r="J27" s="4"/>
       <c r="K27" s="4"/>
@@ -2050,30 +2198,24 @@
       <c r="Z27" s="4"/>
     </row>
     <row r="28" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="9">
-        <v>46289</v>
+      <c r="A28" s="14">
+        <v>46287</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>14</v>
+        <v>64</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F28" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="7"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
       <c r="K28" s="4"/>
@@ -2094,14 +2236,14 @@
       <c r="Z28" s="4"/>
     </row>
     <row r="29" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="9">
-        <v>46289</v>
+      <c r="A29" s="14">
+        <v>46287</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>2</v>
@@ -2109,15 +2251,9 @@
       <c r="E29" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F29" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>18</v>
-      </c>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="7"/>
       <c r="I29" s="4"/>
       <c r="J29" s="4"/>
       <c r="K29" s="4"/>
@@ -2138,30 +2274,24 @@
       <c r="Z29" s="4"/>
     </row>
     <row r="30" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="9">
-        <v>46290</v>
+      <c r="A30" s="14">
+        <v>46287</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>19</v>
+        <v>66</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F30" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="7"/>
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
       <c r="K30" s="4"/>
@@ -2182,28 +2312,14 @@
       <c r="Z30" s="4"/>
     </row>
     <row r="31" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="9">
-        <v>46290</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>23</v>
-      </c>
+      <c r="A31" s="14"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
       <c r="F31" s="4"/>
-      <c r="G31" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>22</v>
-      </c>
+      <c r="G31" s="4"/>
+      <c r="H31" s="7"/>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
       <c r="K31" s="4"/>
@@ -2224,7 +2340,7 @@
       <c r="Z31" s="4"/>
     </row>
     <row r="32" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="8"/>
+      <c r="A32" s="14"/>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
@@ -2252,7 +2368,7 @@
       <c r="Z32" s="4"/>
     </row>
     <row r="33" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="8"/>
+      <c r="A33" s="14"/>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
@@ -2280,7 +2396,7 @@
       <c r="Z33" s="4"/>
     </row>
     <row r="34" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="8"/>
+      <c r="A34" s="14"/>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -2308,7 +2424,7 @@
       <c r="Z34" s="4"/>
     </row>
     <row r="35" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="8"/>
+      <c r="A35" s="14"/>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
@@ -2336,7 +2452,7 @@
       <c r="Z35" s="4"/>
     </row>
     <row r="36" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="8"/>
+      <c r="A36" s="14"/>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4"/>
@@ -2364,7 +2480,7 @@
       <c r="Z36" s="4"/>
     </row>
     <row r="37" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="8"/>
+      <c r="A37" s="14"/>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -2392,14 +2508,30 @@
       <c r="Z37" s="4"/>
     </row>
     <row r="38" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="8"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="7"/>
+      <c r="A38" s="9">
+        <v>46289</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H38" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
@@ -2420,14 +2552,30 @@
       <c r="Z38" s="4"/>
     </row>
     <row r="39" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="8"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
-      <c r="F39" s="4"/>
-      <c r="G39" s="4"/>
-      <c r="H39" s="7"/>
+      <c r="A39" s="9">
+        <v>46289</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
@@ -2448,14 +2596,30 @@
       <c r="Z39" s="4"/>
     </row>
     <row r="40" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="8"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
-      <c r="H40" s="7"/>
+      <c r="A40" s="9">
+        <v>46289</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G40" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
@@ -2476,14 +2640,30 @@
       <c r="Z40" s="4"/>
     </row>
     <row r="41" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="8"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="7"/>
+      <c r="A41" s="9">
+        <v>46290</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>12</v>
+      </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
@@ -2504,14 +2684,28 @@
       <c r="Z41" s="4"/>
     </row>
     <row r="42" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="8"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
-      <c r="E42" s="4"/>
+      <c r="A42" s="9">
+        <v>46290</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F42" s="4"/>
-      <c r="G42" s="4"/>
-      <c r="H42" s="7"/>
+      <c r="G42" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H42" s="10" t="s">
+        <v>22</v>
+      </c>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
@@ -2672,14 +2866,14 @@
       <c r="Z47" s="4"/>
     </row>
     <row r="48" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="11"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12"/>
-      <c r="G48" s="12"/>
-      <c r="H48" s="13"/>
+      <c r="A48" s="8"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="7"/>
       <c r="I48" s="4"/>
       <c r="J48" s="4"/>
       <c r="K48" s="4"/>
@@ -2700,14 +2894,14 @@
       <c r="Z48" s="4"/>
     </row>
     <row r="49" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="4"/>
+      <c r="A49" s="8"/>
       <c r="B49" s="4"/>
       <c r="C49" s="4"/>
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
+      <c r="H49" s="7"/>
       <c r="I49" s="4"/>
       <c r="J49" s="4"/>
       <c r="K49" s="4"/>
@@ -2728,14 +2922,14 @@
       <c r="Z49" s="4"/>
     </row>
     <row r="50" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="4"/>
+      <c r="A50" s="8"/>
       <c r="B50" s="4"/>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
+      <c r="H50" s="7"/>
       <c r="I50" s="4"/>
       <c r="J50" s="4"/>
       <c r="K50" s="4"/>
@@ -2756,14 +2950,14 @@
       <c r="Z50" s="4"/>
     </row>
     <row r="51" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="4"/>
+      <c r="A51" s="8"/>
       <c r="B51" s="4"/>
       <c r="C51" s="4"/>
       <c r="D51" s="4"/>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
+      <c r="H51" s="7"/>
       <c r="I51" s="4"/>
       <c r="J51" s="4"/>
       <c r="K51" s="4"/>
@@ -2784,14 +2978,14 @@
       <c r="Z51" s="4"/>
     </row>
     <row r="52" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="4"/>
+      <c r="A52" s="8"/>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
+      <c r="H52" s="7"/>
       <c r="I52" s="4"/>
       <c r="J52" s="4"/>
       <c r="K52" s="4"/>
@@ -2812,14 +3006,14 @@
       <c r="Z52" s="4"/>
     </row>
     <row r="53" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="4"/>
+      <c r="A53" s="8"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
+      <c r="H53" s="7"/>
       <c r="I53" s="4"/>
       <c r="J53" s="4"/>
       <c r="K53" s="4"/>
@@ -2840,14 +3034,14 @@
       <c r="Z53" s="4"/>
     </row>
     <row r="54" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="4"/>
+      <c r="A54" s="8"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
+      <c r="H54" s="7"/>
       <c r="I54" s="4"/>
       <c r="J54" s="4"/>
       <c r="K54" s="4"/>
@@ -2868,14 +3062,14 @@
       <c r="Z54" s="4"/>
     </row>
     <row r="55" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="4"/>
+      <c r="A55" s="8"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
       <c r="D55" s="4"/>
       <c r="E55" s="4"/>
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
+      <c r="H55" s="7"/>
       <c r="I55" s="4"/>
       <c r="J55" s="4"/>
       <c r="K55" s="4"/>
@@ -2896,14 +3090,14 @@
       <c r="Z55" s="4"/>
     </row>
     <row r="56" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="4"/>
+      <c r="A56" s="8"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
       <c r="D56" s="4"/>
       <c r="E56" s="4"/>
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
+      <c r="H56" s="7"/>
       <c r="I56" s="4"/>
       <c r="J56" s="4"/>
       <c r="K56" s="4"/>
@@ -2924,14 +3118,14 @@
       <c r="Z56" s="4"/>
     </row>
     <row r="57" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="4"/>
+      <c r="A57" s="8"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
       <c r="F57" s="4"/>
       <c r="G57" s="4"/>
-      <c r="H57" s="4"/>
+      <c r="H57" s="7"/>
       <c r="I57" s="4"/>
       <c r="J57" s="4"/>
       <c r="K57" s="4"/>
@@ -2952,14 +3146,14 @@
       <c r="Z57" s="4"/>
     </row>
     <row r="58" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="4"/>
+      <c r="A58" s="8"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
+      <c r="H58" s="7"/>
       <c r="I58" s="4"/>
       <c r="J58" s="4"/>
       <c r="K58" s="4"/>
@@ -2980,14 +3174,14 @@
       <c r="Z58" s="4"/>
     </row>
     <row r="59" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
-      <c r="F59" s="4"/>
-      <c r="G59" s="4"/>
-      <c r="H59" s="4"/>
+      <c r="A59" s="11"/>
+      <c r="B59" s="12"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="12"/>
+      <c r="H59" s="13"/>
       <c r="I59" s="4"/>
       <c r="J59" s="4"/>
       <c r="K59" s="4"/>
@@ -29495,6 +29689,116 @@
       <c r="G1014" s="4"/>
       <c r="H1014" s="4"/>
     </row>
+    <row r="1015" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1015" s="4"/>
+      <c r="B1015" s="4"/>
+      <c r="C1015" s="4"/>
+      <c r="D1015" s="4"/>
+      <c r="E1015" s="4"/>
+      <c r="F1015" s="4"/>
+      <c r="G1015" s="4"/>
+      <c r="H1015" s="4"/>
+    </row>
+    <row r="1016" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1016" s="4"/>
+      <c r="B1016" s="4"/>
+      <c r="C1016" s="4"/>
+      <c r="D1016" s="4"/>
+      <c r="E1016" s="4"/>
+      <c r="F1016" s="4"/>
+      <c r="G1016" s="4"/>
+      <c r="H1016" s="4"/>
+    </row>
+    <row r="1017" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1017" s="4"/>
+      <c r="B1017" s="4"/>
+      <c r="C1017" s="4"/>
+      <c r="D1017" s="4"/>
+      <c r="E1017" s="4"/>
+      <c r="F1017" s="4"/>
+      <c r="G1017" s="4"/>
+      <c r="H1017" s="4"/>
+    </row>
+    <row r="1018" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1018" s="4"/>
+      <c r="B1018" s="4"/>
+      <c r="C1018" s="4"/>
+      <c r="D1018" s="4"/>
+      <c r="E1018" s="4"/>
+      <c r="F1018" s="4"/>
+      <c r="G1018" s="4"/>
+      <c r="H1018" s="4"/>
+    </row>
+    <row r="1019" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1019" s="4"/>
+      <c r="B1019" s="4"/>
+      <c r="C1019" s="4"/>
+      <c r="D1019" s="4"/>
+      <c r="E1019" s="4"/>
+      <c r="F1019" s="4"/>
+      <c r="G1019" s="4"/>
+      <c r="H1019" s="4"/>
+    </row>
+    <row r="1020" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1020" s="4"/>
+      <c r="B1020" s="4"/>
+      <c r="C1020" s="4"/>
+      <c r="D1020" s="4"/>
+      <c r="E1020" s="4"/>
+      <c r="F1020" s="4"/>
+      <c r="G1020" s="4"/>
+      <c r="H1020" s="4"/>
+    </row>
+    <row r="1021" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1021" s="4"/>
+      <c r="B1021" s="4"/>
+      <c r="C1021" s="4"/>
+      <c r="D1021" s="4"/>
+      <c r="E1021" s="4"/>
+      <c r="F1021" s="4"/>
+      <c r="G1021" s="4"/>
+      <c r="H1021" s="4"/>
+    </row>
+    <row r="1022" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1022" s="4"/>
+      <c r="B1022" s="4"/>
+      <c r="C1022" s="4"/>
+      <c r="D1022" s="4"/>
+      <c r="E1022" s="4"/>
+      <c r="F1022" s="4"/>
+      <c r="G1022" s="4"/>
+      <c r="H1022" s="4"/>
+    </row>
+    <row r="1023" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1023" s="4"/>
+      <c r="B1023" s="4"/>
+      <c r="C1023" s="4"/>
+      <c r="D1023" s="4"/>
+      <c r="E1023" s="4"/>
+      <c r="F1023" s="4"/>
+      <c r="G1023" s="4"/>
+      <c r="H1023" s="4"/>
+    </row>
+    <row r="1024" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1024" s="4"/>
+      <c r="B1024" s="4"/>
+      <c r="C1024" s="4"/>
+      <c r="D1024" s="4"/>
+      <c r="E1024" s="4"/>
+      <c r="F1024" s="4"/>
+      <c r="G1024" s="4"/>
+      <c r="H1024" s="4"/>
+    </row>
+    <row r="1025" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1025" s="4"/>
+      <c r="B1025" s="4"/>
+      <c r="C1025" s="4"/>
+      <c r="D1025" s="4"/>
+      <c r="E1025" s="4"/>
+      <c r="F1025" s="4"/>
+      <c r="G1025" s="4"/>
+      <c r="H1025" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Moved the Practice question folder from 3rd-week folder to its parent folder
</commit_message>
<xml_diff>
--- a/Dyashin-Training-Master-Tracker-Record.xlsx
+++ b/Dyashin-Training-Master-Tracker-Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dyashin-tutorial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A855CB-F68B-415B-9B17-2479F2D2AD7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E05EC9F6-D168-49E4-B5F8-9C093A4B3E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{04FCAFE5-9534-4F2F-ACC7-2F9728B33BA2}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="75">
   <si>
     <t>Date</t>
   </si>
@@ -237,7 +237,28 @@
     <t>Completed Assignment task 2.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Task </t>
+    <t>Practiced Function methods</t>
+  </si>
+  <si>
+    <t>Learnt Prototype Inheritance, debouncing &amp; thortling</t>
+  </si>
+  <si>
+    <t>Completed Basic questions of JS practice questions provided</t>
+  </si>
+  <si>
+    <t>Written the Assessment given</t>
+  </si>
+  <si>
+    <t>Completed Assignment task 2.3</t>
+  </si>
+  <si>
+    <t>Practice Event Propogation</t>
+  </si>
+  <si>
+    <t>Made the Time Clock task dynamic using JS</t>
+  </si>
+  <si>
+    <t>Completed Assignment 2.4 all questions</t>
   </si>
 </sst>
 </file>
@@ -2246,7 +2267,7 @@
         <v>65</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>23</v>
@@ -2284,7 +2305,7 @@
         <v>66</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>67</v>
+        <v>9</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>23</v>
@@ -2312,11 +2333,21 @@
       <c r="Z30" s="4"/>
     </row>
     <row r="31" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="14"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="A31" s="14">
+        <v>46288</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="7"/>
@@ -2340,11 +2371,21 @@
       <c r="Z31" s="4"/>
     </row>
     <row r="32" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="14"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
+      <c r="A32" s="14">
+        <v>46288</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="7"/>
@@ -2368,11 +2409,21 @@
       <c r="Z32" s="4"/>
     </row>
     <row r="33" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="14"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
+      <c r="A33" s="14">
+        <v>46289</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="7"/>
@@ -2395,12 +2446,22 @@
       <c r="Y33" s="4"/>
       <c r="Z33" s="4"/>
     </row>
-    <row r="34" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="14"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
+    <row r="34" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="14">
+        <v>46288</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
       <c r="H34" s="7"/>
@@ -2424,11 +2485,21 @@
       <c r="Z34" s="4"/>
     </row>
     <row r="35" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="14"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
+      <c r="A35" s="14">
+        <v>46288</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="7"/>
@@ -2726,11 +2797,21 @@
       <c r="Z42" s="4"/>
     </row>
     <row r="43" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="8"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
-      <c r="E43" s="4"/>
+      <c r="A43" s="14">
+        <v>46290</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="7"/>
@@ -2753,12 +2834,22 @@
       <c r="Y43" s="4"/>
       <c r="Z43" s="4"/>
     </row>
-    <row r="44" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="8"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
-      <c r="E44" s="4"/>
+    <row r="44" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="14">
+        <v>46290</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="7"/>
@@ -2781,12 +2872,22 @@
       <c r="Y44" s="4"/>
       <c r="Z44" s="4"/>
     </row>
-    <row r="45" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="8"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
-      <c r="E45" s="4"/>
+    <row r="45" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="14">
+        <v>46290</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="7"/>
@@ -2809,12 +2910,22 @@
       <c r="Y45" s="4"/>
       <c r="Z45" s="4"/>
     </row>
-    <row r="46" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="8"/>
-      <c r="B46" s="4"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+    <row r="46" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="14">
+        <v>46290</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="7"/>

</xml_diff>

<commit_message>
updated excel record file
</commit_message>
<xml_diff>
--- a/Dyashin-Training-Master-Tracker-Record.xlsx
+++ b/Dyashin-Training-Master-Tracker-Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dyashin-tutorial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E05EC9F6-D168-49E4-B5F8-9C093A4B3E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B2FFB1D-7BCD-47E9-8E48-6319E4D348E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{04FCAFE5-9534-4F2F-ACC7-2F9728B33BA2}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="82">
   <si>
     <t>Date</t>
   </si>
@@ -60,13 +60,7 @@
     <t>JavaScript</t>
   </si>
   <si>
-    <t>Digital Clock</t>
-  </si>
-  <si>
     <t>Assignment</t>
-  </si>
-  <si>
-    <t>Link</t>
   </si>
   <si>
     <t>S3</t>
@@ -90,9 +84,6 @@
     <t>Responsive UI</t>
   </si>
   <si>
-    <t>Good</t>
-  </si>
-  <si>
     <t>Callbacks</t>
   </si>
   <si>
@@ -100,9 +91,6 @@
   </si>
   <si>
     <t>Promise exercises</t>
-  </si>
-  <si>
-    <t>Need improvement</t>
   </si>
   <si>
     <t>COMPLETED</t>
@@ -260,12 +248,45 @@
   <si>
     <t>Completed Assignment 2.4 all questions</t>
   </si>
+  <si>
+    <t>Digital Clock Deployment</t>
+  </si>
+  <si>
+    <t>http://time-shower-bucket.s3-website.ap-south-1.amazonaws.com/</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/blob/main/3rd-week/16th-day/Funtion%20methods.html</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/blob/main/3rd-week/16th-day/Prototype-inheritance.html</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/blob/main/3rd-week/Practice%20questions/JavaScript%20Practice%20Questions%20Answers.docx</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/tree/main/Practice%20questions</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/blob/main/1st-week/4th-day-css/notes.txt</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/blob/main/1st-week/4th-day-css/CSS/task.html</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/blob/main/1st-week/5th-day-css/position.html</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/blob/main/1st-week/5th-day-css/animation.html</t>
+  </si>
+  <si>
+    <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/tree/main/1st-week/5th-day-css/case-study-task</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,6 +313,14 @@
       <color theme="0"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -428,10 +457,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -473,8 +503,12 @@
     <xf numFmtId="16" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
@@ -890,8 +924,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41E48F9C-D00C-4230-BFD8-0CECC030125D}" name="Table1" displayName="Table1" ref="A1:H59" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11" tableBorderDxfId="9" totalsRowBorderDxfId="8">
-  <autoFilter ref="A1:H59" xr:uid="{41E48F9C-D00C-4230-BFD8-0CECC030125D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41E48F9C-D00C-4230-BFD8-0CECC030125D}" name="Table1" displayName="Table1" ref="A1:H57" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+  <autoFilter ref="A1:H57" xr:uid="{41E48F9C-D00C-4230-BFD8-0CECC030125D}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{2A26C5F3-F6F5-408A-9023-BEE119F726B8}" name="Date" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{EFAA7E6B-D8D1-4A29-ADAB-AE44D9FE76A7}" name="Topic" dataDxfId="6"/>
@@ -1203,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C217E04-B9EA-4E6C-A4A3-4C970AA68344}">
-  <dimension ref="A1:Z1025"/>
+  <dimension ref="A1:Z1023"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="20.7109375" style="5" customWidth="1"/>
@@ -1237,7 +1271,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
@@ -1291,16 +1325,16 @@
         <v>46267</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
@@ -1329,16 +1363,16 @@
         <v>46268</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -1367,16 +1401,16 @@
         <v>46269</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -1405,16 +1439,16 @@
         <v>46269</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -1443,16 +1477,16 @@
         <v>46272</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -1476,23 +1510,25 @@
       <c r="Y7" s="4"/>
       <c r="Z7" s="4"/>
     </row>
-    <row r="8" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>46273</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F8" s="4"/>
+      <c r="F8" s="15" t="s">
+        <v>77</v>
+      </c>
       <c r="G8" s="4"/>
       <c r="H8" s="7"/>
       <c r="I8" s="4"/>
@@ -1514,23 +1550,25 @@
       <c r="Y8" s="4"/>
       <c r="Z8" s="4"/>
     </row>
-    <row r="9" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>46273</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F9" s="4"/>
+      <c r="F9" s="15" t="s">
+        <v>78</v>
+      </c>
       <c r="G9" s="4"/>
       <c r="H9" s="7"/>
       <c r="I9" s="4"/>
@@ -1557,21 +1595,21 @@
         <v>46273</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -1592,23 +1630,25 @@
       <c r="Y10" s="4"/>
       <c r="Z10" s="4"/>
     </row>
-    <row r="11" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>46274</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F11" s="4"/>
+      <c r="F11" s="15" t="s">
+        <v>79</v>
+      </c>
       <c r="G11" s="4"/>
       <c r="H11" s="7"/>
       <c r="I11" s="4"/>
@@ -1630,23 +1670,25 @@
       <c r="Y11" s="4"/>
       <c r="Z11" s="4"/>
     </row>
-    <row r="12" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14">
         <v>46274</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F12" s="4"/>
+      <c r="F12" s="15" t="s">
+        <v>80</v>
+      </c>
       <c r="G12" s="4"/>
       <c r="H12" s="7"/>
       <c r="I12" s="4"/>
@@ -1668,23 +1710,25 @@
       <c r="Y12" s="4"/>
       <c r="Z12" s="4"/>
     </row>
-    <row r="13" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>46274</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F13" s="4"/>
+      <c r="F13" s="15" t="s">
+        <v>81</v>
+      </c>
       <c r="G13" s="4"/>
       <c r="H13" s="7"/>
       <c r="I13" s="4"/>
@@ -1711,16 +1755,16 @@
         <v>46275</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -1749,16 +1793,16 @@
         <v>46276</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1787,16 +1831,16 @@
         <v>46276</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -1856,13 +1900,13 @@
         <v>7</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1894,13 +1938,13 @@
         <v>7</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1932,13 +1976,13 @@
         <v>7</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -1970,13 +2014,13 @@
         <v>7</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -2008,13 +2052,13 @@
         <v>7</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -2046,13 +2090,13 @@
         <v>7</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -2084,13 +2128,13 @@
         <v>7</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -2150,13 +2194,13 @@
         <v>7</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -2188,13 +2232,13 @@
         <v>7</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -2226,13 +2270,13 @@
         <v>7</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -2264,13 +2308,13 @@
         <v>7</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -2302,13 +2346,13 @@
         <v>7</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -2340,13 +2384,13 @@
         <v>7</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -2378,13 +2422,13 @@
         <v>7</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -2416,13 +2460,13 @@
         <v>7</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -2448,19 +2492,19 @@
     </row>
     <row r="34" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="14">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -2486,19 +2530,19 @@
     </row>
     <row r="35" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="14">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -2522,14 +2566,28 @@
       <c r="Y35" s="4"/>
       <c r="Z35" s="4"/>
     </row>
-    <row r="36" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="14"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
+    <row r="36" spans="1:26" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="9">
+        <v>46289</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="H36" s="7"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
@@ -2551,13 +2609,25 @@
       <c r="Z36" s="4"/>
     </row>
     <row r="37" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="14"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="A37" s="9">
+        <v>46289</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
+      <c r="G37" s="4" t="s">
+        <v>10</v>
+      </c>
       <c r="H37" s="7"/>
       <c r="I37" s="4"/>
       <c r="J37" s="4"/>
@@ -2579,30 +2649,26 @@
       <c r="Z37" s="4"/>
     </row>
     <row r="38" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="9">
+      <c r="A38" s="14">
         <v>46289</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F38" s="4"/>
+      <c r="G38" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G38" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="H38" s="7"/>
       <c r="I38" s="4"/>
       <c r="J38" s="4"/>
       <c r="K38" s="4"/>
@@ -2624,29 +2690,25 @@
     </row>
     <row r="39" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="9">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="F39" s="4"/>
+      <c r="G39" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G39" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="H39" s="7"/>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
       <c r="K39" s="4"/>
@@ -2668,29 +2730,25 @@
     </row>
     <row r="40" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="9">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="F40" s="4"/>
+      <c r="G40" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G40" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>18</v>
-      </c>
+      <c r="H40" s="10"/>
       <c r="I40" s="4"/>
       <c r="J40" s="4"/>
       <c r="K40" s="4"/>
@@ -2710,31 +2768,27 @@
       <c r="Y40" s="4"/>
       <c r="Z40" s="4"/>
     </row>
-    <row r="41" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="9">
+    <row r="41" spans="1:26" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="14">
         <v>46290</v>
       </c>
       <c r="B41" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D41" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="E41" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>20</v>
+      <c r="F41" s="15" t="s">
+        <v>73</v>
       </c>
-      <c r="E41" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>12</v>
-      </c>
+      <c r="G41" s="4"/>
+      <c r="H41" s="7"/>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4"/>
@@ -2754,29 +2808,27 @@
       <c r="Y41" s="4"/>
       <c r="Z41" s="4"/>
     </row>
-    <row r="42" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="9">
+    <row r="42" spans="1:26" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="14">
         <v>46290</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>21</v>
+        <v>64</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F42" s="4"/>
-      <c r="G42" s="4" t="s">
-        <v>12</v>
+      <c r="F42" s="15" t="s">
+        <v>74</v>
       </c>
-      <c r="H42" s="10" t="s">
-        <v>22</v>
-      </c>
+      <c r="G42" s="4"/>
+      <c r="H42" s="7"/>
       <c r="I42" s="4"/>
       <c r="J42" s="4"/>
       <c r="K42" s="4"/>
@@ -2796,23 +2848,25 @@
       <c r="Y42" s="4"/>
       <c r="Z42" s="4"/>
     </row>
-    <row r="43" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:26" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="14">
         <v>46290</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F43" s="4"/>
+      <c r="F43" s="15" t="s">
+        <v>75</v>
+      </c>
       <c r="G43" s="4"/>
       <c r="H43" s="7"/>
       <c r="I43" s="4"/>
@@ -2834,23 +2888,25 @@
       <c r="Y43" s="4"/>
       <c r="Z43" s="4"/>
     </row>
-    <row r="44" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:26" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="14">
         <v>46290</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="F44" s="4"/>
+      <c r="F44" s="15" t="s">
+        <v>76</v>
+      </c>
       <c r="G44" s="4"/>
       <c r="H44" s="7"/>
       <c r="I44" s="4"/>
@@ -2872,22 +2928,12 @@
       <c r="Y44" s="4"/>
       <c r="Z44" s="4"/>
     </row>
-    <row r="45" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="14">
-        <v>46290</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>23</v>
-      </c>
+    <row r="45" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="8"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="7"/>
@@ -2910,22 +2956,12 @@
       <c r="Y45" s="4"/>
       <c r="Z45" s="4"/>
     </row>
-    <row r="46" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="14">
-        <v>46290</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>23</v>
-      </c>
+    <row r="46" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="8"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="7"/>
@@ -3229,14 +3265,14 @@
       <c r="Z56" s="4"/>
     </row>
     <row r="57" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="8"/>
-      <c r="B57" s="4"/>
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="G57" s="4"/>
-      <c r="H57" s="7"/>
+      <c r="A57" s="11"/>
+      <c r="B57" s="12"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="13"/>
       <c r="I57" s="4"/>
       <c r="J57" s="4"/>
       <c r="K57" s="4"/>
@@ -3257,14 +3293,14 @@
       <c r="Z57" s="4"/>
     </row>
     <row r="58" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="8"/>
+      <c r="A58" s="4"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
       <c r="F58" s="4"/>
       <c r="G58" s="4"/>
-      <c r="H58" s="7"/>
+      <c r="H58" s="4"/>
       <c r="I58" s="4"/>
       <c r="J58" s="4"/>
       <c r="K58" s="4"/>
@@ -3285,14 +3321,14 @@
       <c r="Z58" s="4"/>
     </row>
     <row r="59" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="11"/>
-      <c r="B59" s="12"/>
-      <c r="C59" s="12"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="12"/>
-      <c r="F59" s="12"/>
-      <c r="G59" s="12"/>
-      <c r="H59" s="13"/>
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+      <c r="F59" s="4"/>
+      <c r="G59" s="4"/>
+      <c r="H59" s="4"/>
       <c r="I59" s="4"/>
       <c r="J59" s="4"/>
       <c r="K59" s="4"/>
@@ -29890,30 +29926,22 @@
       <c r="G1023" s="4"/>
       <c r="H1023" s="4"/>
     </row>
-    <row r="1024" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1024" s="4"/>
-      <c r="B1024" s="4"/>
-      <c r="C1024" s="4"/>
-      <c r="D1024" s="4"/>
-      <c r="E1024" s="4"/>
-      <c r="F1024" s="4"/>
-      <c r="G1024" s="4"/>
-      <c r="H1024" s="4"/>
-    </row>
-    <row r="1025" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1025" s="4"/>
-      <c r="B1025" s="4"/>
-      <c r="C1025" s="4"/>
-      <c r="D1025" s="4"/>
-      <c r="E1025" s="4"/>
-      <c r="F1025" s="4"/>
-      <c r="G1025" s="4"/>
-      <c r="H1025" s="4"/>
-    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F36" r:id="rId1" xr:uid="{40D2E850-5216-4D06-BCF9-E8A291270CA7}"/>
+    <hyperlink ref="F41" r:id="rId2" xr:uid="{02EBE818-8C77-441B-B784-7544B58B73EA}"/>
+    <hyperlink ref="F42" r:id="rId3" xr:uid="{D14828DD-45B1-40B4-945F-18CE1A549F52}"/>
+    <hyperlink ref="F43" r:id="rId4" xr:uid="{1C953428-C32A-4BE7-8CA6-C196F9044F96}"/>
+    <hyperlink ref="F44" r:id="rId5" xr:uid="{6D894DD0-66F1-4FCB-89BC-510AE017F863}"/>
+    <hyperlink ref="F8" r:id="rId6" xr:uid="{4665259C-60AE-4261-9B5C-F53536EC4A24}"/>
+    <hyperlink ref="F9" r:id="rId7" xr:uid="{63347461-6B60-4BC7-BBFF-9E8A4FBEF590}"/>
+    <hyperlink ref="F11" r:id="rId8" xr:uid="{536537D0-0699-47E0-BFBE-44E93C63BEE6}"/>
+    <hyperlink ref="F12" r:id="rId9" xr:uid="{54DD8B9D-0DB3-4059-9AB8-6715995F5096}"/>
+    <hyperlink ref="F13" r:id="rId10" xr:uid="{85FD4687-67FA-4D02-84DC-5499077AB5ED}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Created 4th week folder and 17th-day notes
</commit_message>
<xml_diff>
--- a/Dyashin-Training-Master-Tracker-Record.xlsx
+++ b/Dyashin-Training-Master-Tracker-Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dyashin-tutorial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B2FFB1D-7BCD-47E9-8E48-6319E4D348E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B51F5B1-0045-41F8-9A43-A17EFEEDA17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{04FCAFE5-9534-4F2F-ACC7-2F9728B33BA2}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="85">
   <si>
     <t>Date</t>
   </si>
@@ -67,9 +67,6 @@
   </si>
   <si>
     <t>—</t>
-  </si>
-  <si>
-    <t>JS</t>
   </si>
   <si>
     <t>Array problems</t>
@@ -280,6 +277,18 @@
   </si>
   <si>
     <t>https://github.com/Jnbhuvan/Dyashin_Training_Repo/tree/main/1st-week/5th-day-css/case-study-task</t>
+  </si>
+  <si>
+    <t>HTML, CSS, JS</t>
+  </si>
+  <si>
+    <t>Completed Half of the Case Study task Given</t>
+  </si>
+  <si>
+    <t>Half</t>
+  </si>
+  <si>
+    <t>Completed the Rest of the JS Q&amp;A Given</t>
   </si>
 </sst>
 </file>
@@ -1271,7 +1280,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
@@ -1325,16 +1334,16 @@
         <v>46267</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
@@ -1363,16 +1372,16 @@
         <v>46268</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>25</v>
-      </c>
       <c r="E4" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
@@ -1401,16 +1410,16 @@
         <v>46269</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
@@ -1439,16 +1448,16 @@
         <v>46269</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
@@ -1477,16 +1486,16 @@
         <v>46272</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
@@ -1515,19 +1524,19 @@
         <v>46273</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>31</v>
-      </c>
       <c r="E8" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="7"/>
@@ -1555,19 +1564,19 @@
         <v>46273</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="7"/>
@@ -1595,21 +1604,21 @@
         <v>46273</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>34</v>
-      </c>
       <c r="D10" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
       <c r="H10" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
@@ -1635,19 +1644,19 @@
         <v>46274</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="D11" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="7"/>
@@ -1675,19 +1684,19 @@
         <v>46274</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="7"/>
@@ -1715,19 +1724,19 @@
         <v>46274</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="E13" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="7"/>
@@ -1755,16 +1764,16 @@
         <v>46275</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>45</v>
-      </c>
       <c r="D14" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -1793,16 +1802,16 @@
         <v>46276</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>47</v>
-      </c>
       <c r="D15" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1831,16 +1840,16 @@
         <v>46276</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>50</v>
-      </c>
       <c r="E16" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -1900,13 +1909,13 @@
         <v>7</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
@@ -1938,13 +1947,13 @@
         <v>7</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
@@ -1976,13 +1985,13 @@
         <v>7</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
@@ -2014,13 +2023,13 @@
         <v>7</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
@@ -2052,13 +2061,13 @@
         <v>7</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
@@ -2090,13 +2099,13 @@
         <v>7</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
@@ -2128,13 +2137,13 @@
         <v>7</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
@@ -2194,13 +2203,13 @@
         <v>7</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F26" s="4"/>
       <c r="G26" s="4"/>
@@ -2232,13 +2241,13 @@
         <v>7</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
@@ -2270,13 +2279,13 @@
         <v>7</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
@@ -2308,13 +2317,13 @@
         <v>7</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
@@ -2346,13 +2355,13 @@
         <v>7</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
@@ -2384,13 +2393,13 @@
         <v>7</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
@@ -2422,13 +2431,13 @@
         <v>7</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -2460,13 +2469,13 @@
         <v>7</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
@@ -2498,13 +2507,13 @@
         <v>7</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F34" s="4"/>
       <c r="G34" s="4"/>
@@ -2536,13 +2545,13 @@
         <v>7</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F35" s="4"/>
       <c r="G35" s="4"/>
@@ -2574,16 +2583,16 @@
         <v>7</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G36" s="4" t="s">
         <v>9</v>
@@ -2613,16 +2622,16 @@
         <v>46289</v>
       </c>
       <c r="B37" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C37" s="4" t="s">
+      <c r="D37" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D37" s="4" t="s">
-        <v>13</v>
-      </c>
       <c r="E37" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F37" s="4"/>
       <c r="G37" s="4" t="s">
@@ -2653,16 +2662,16 @@
         <v>46289</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D38" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F38" s="4"/>
       <c r="G38" s="4" t="s">
@@ -2693,16 +2702,16 @@
         <v>46290</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C39" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D39" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D39" s="4" t="s">
-        <v>17</v>
-      </c>
       <c r="E39" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4" t="s">
@@ -2733,16 +2742,16 @@
         <v>46290</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F40" s="4"/>
       <c r="G40" s="4" t="s">
@@ -2773,19 +2782,19 @@
         <v>46290</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F41" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G41" s="4"/>
       <c r="H41" s="7"/>
@@ -2813,19 +2822,19 @@
         <v>46290</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F42" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G42" s="4"/>
       <c r="H42" s="7"/>
@@ -2853,19 +2862,19 @@
         <v>46290</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D43" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G43" s="4"/>
       <c r="H43" s="7"/>
@@ -2893,19 +2902,19 @@
         <v>46290</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D44" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G44" s="4"/>
       <c r="H44" s="7"/>
@@ -2956,12 +2965,22 @@
       <c r="Y45" s="4"/>
       <c r="Z45" s="4"/>
     </row>
-    <row r="46" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="8"/>
-      <c r="B46" s="4"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+    <row r="46" spans="1:26" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="14">
+        <v>46293</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="7"/>
@@ -2985,11 +3004,21 @@
       <c r="Z46" s="4"/>
     </row>
     <row r="47" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="8"/>
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
+      <c r="A47" s="14">
+        <v>46293</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="7"/>
@@ -3013,8 +3042,12 @@
       <c r="Z47" s="4"/>
     </row>
     <row r="48" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="8"/>
-      <c r="B48" s="4"/>
+      <c r="A48" s="14">
+        <v>46294</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>81</v>
+      </c>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>

</xml_diff>

<commit_message>
Updated the master tracker excel
</commit_message>
<xml_diff>
--- a/Dyashin-Training-Master-Tracker-Record.xlsx
+++ b/Dyashin-Training-Master-Tracker-Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\dyashin-tutorial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B51F5B1-0045-41F8-9A43-A17EFEEDA17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BD3271-5B97-4DC3-BF9C-B0EEF2616663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{04FCAFE5-9534-4F2F-ACC7-2F9728B33BA2}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="87">
   <si>
     <t>Date</t>
   </si>
@@ -289,6 +289,12 @@
   </si>
   <si>
     <t>Completed the Rest of the JS Q&amp;A Given</t>
+  </si>
+  <si>
+    <t>Continued Case study task given</t>
+  </si>
+  <si>
+    <t>Continued completion of JS Q&amp;A Given</t>
   </si>
 </sst>
 </file>
@@ -3048,9 +3054,15 @@
       <c r="B48" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
-      <c r="E48" s="4"/>
+      <c r="C48" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="7"/>
@@ -3074,11 +3086,21 @@
       <c r="Z48" s="4"/>
     </row>
     <row r="49" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="8"/>
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
+      <c r="A49" s="14">
+        <v>46294</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>83</v>
+      </c>
       <c r="F49" s="4"/>
       <c r="G49" s="4"/>
       <c r="H49" s="7"/>
@@ -3102,8 +3124,12 @@
       <c r="Z49" s="4"/>
     </row>
     <row r="50" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="8"/>
-      <c r="B50" s="4"/>
+      <c r="A50" s="14">
+        <v>46295</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>81</v>
+      </c>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
       <c r="E50" s="4"/>

</xml_diff>